<commit_message>
Rev. C: genel aydınlatma V3 — 17 × BLADE 12 bölge bazlı; tüm görseller + 360° yenilendi (video yok)
</commit_message>
<xml_diff>
--- a/Malzeme_Listesi.xlsx
+++ b/Malzeme_Listesi.xlsx
@@ -469,7 +469,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Kuyumcu Mağazası · Aydınlatma Malzeme Listesi · GMC LED · 17 Ekim 2026 · Rev. B</t>
+          <t>Kuyumcu Mağazası · Aydınlatma Malzeme Listesi · GMC LED · 17 Ekim 2026 · Rev. C</t>
         </is>
       </c>
     </row>
@@ -578,13 +578,13 @@
         </is>
       </c>
       <c r="E5" s="3" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>21</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>189</v>
+        <v>357</v>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
       <c r="I5" s="3">
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="F11" s="3" t="inlineStr"/>
       <c r="G11" s="3" t="inlineStr"/>
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1553</v>
+        <v>1721</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -978,7 +978,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>404</v>
+        <v>447</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1817</v>
+        <v>2014</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1008,7 +1008,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>21804</v>
+        <v>24163</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>

</xml_diff>